<commit_message>
Sync poultry finmodel with rabbit baseline: NPV/IRR, financing, KPI docs
- Update finmodel xlsx: CAPEX balance (solar+compost vs biogaz), fertilizer line,
  NPV-IRR sheet (16-year DCF @10%), Financing sheet (FNB/RAL/banks template)
- Fix revenue total refs and CAPEX total row in Economics sheet
- Sync poultry-teo.yaml, registry, T01/T02/T09, appendix 02/03, finmodel-summary
- Add financing-structure.md and sync-poultry-finmodel.py script

Co-authored-by: Demid369 <Demid369@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/teo-poultry/_incoming/finmodel-pticekompleks-12-mlrd.xlsx
+++ b/docs/teo-poultry/_incoming/finmodel-pticekompleks-12-mlrd.xlsx
@@ -15,6 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAPEX" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OPEX" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Экономика" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPV-IRR" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Финансирование" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -30,7 +32,7 @@
     <numFmt numFmtId="167" formatCode="#,##0;\(#,##0\);\-"/>
     <numFmt numFmtId="168" formatCode="#,##0.0;\(#,##0.0\);\-"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -159,8 +161,15 @@
       <family val="0"/>
       <sz val="8"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -183,6 +192,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFD9E5DC"/>
         <bgColor rgb="FFCCCCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -229,7 +243,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="116">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -576,6 +590,12 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -829,7 +849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="40" customWidth="1" style="58" min="1" max="1"/>
@@ -982,7 +1002,7 @@
         </is>
       </c>
       <c r="B16" s="65" t="n">
-        <v>480</v>
+        <v>476</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="59">
@@ -1008,7 +1028,53 @@
     <row r="20" ht="15" customHeight="1" s="59">
       <c r="A20" s="61" t="inlineStr">
         <is>
-          <t>Подробности — на листах: Продукция, Выручка, Корма, CAPEX, OPEX, Экономика, Допущения.</t>
+          <t>NPV @ 10%, млн ₽</t>
+        </is>
+      </c>
+      <c r="B20" s="58">
+        <f>NPV-IRR!B22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="58" t="inlineStr">
+        <is>
+          <t>IRR, %</t>
+        </is>
+      </c>
+      <c r="B21" s="58">
+        <f>NPV-IRR!B23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="58" t="inlineStr">
+        <is>
+          <t>Финансирование</t>
+        </is>
+      </c>
+      <c r="B22" s="58" t="inlineStr">
+        <is>
+          <t>лист «Финансирование»</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="58" t="inlineStr">
+        <is>
+          <t>Энергетика</t>
+        </is>
+      </c>
+      <c r="B23" s="58" t="inlineStr">
+        <is>
+          <t>solar 10 МВт·ч + compost 5 т/ч (= кролики); без лок. biogaz+ГПU</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="58" t="inlineStr">
+        <is>
+          <t>Подробности — листы: Продукция, Выручка, Корма, CAPEX, OPEX, Экономика, NPV-IRR, Финансирование, Допущения.</t>
         </is>
       </c>
     </row>
@@ -1016,6 +1082,415 @@
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" style="59" min="1" max="1"/>
+    <col width="28" customWidth="1" style="59" min="2" max="2"/>
+    <col width="38" customWidth="1" style="59" min="3" max="3"/>
+    <col width="16" customWidth="1" style="59" min="4" max="4"/>
+    <col width="10" customWidth="1" style="59" min="5" max="5"/>
+    <col width="42" customWidth="1" style="59" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="116" t="inlineStr">
+        <is>
+          <t>СТРУКТУРА ФИНАНСИРОВАНИЯ — ПТИЦЕКОМПЛЕКС 12 000 млн ₽</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Шаблон: docs/1.2-слайд Фин модель.xlsx (ФНБ / РАЛ / ФРП / банки) · блок птицы отдельно от APK 100 млрд</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Сумма инвестиций</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>12000</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>млн ₽</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="117" t="inlineStr"/>
+      <c r="B5" s="117" t="inlineStr">
+        <is>
+          <t>Источник</t>
+        </is>
+      </c>
+      <c r="C5" s="117" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="D5" s="117" t="inlineStr">
+        <is>
+          <t>Сумма, млн ₽</t>
+        </is>
+      </c>
+      <c r="E5" s="117" t="inlineStr">
+        <is>
+          <t>Доля</t>
+        </is>
+      </c>
+      <c r="F5" s="117" t="inlineStr">
+        <is>
+          <t>Комментарий</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ФНБ</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Фонд национального благосостояния</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Долевое участие в проекте</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>600</v>
+      </c>
+      <c r="E6">
+        <f>D6/$B$3</f>
+        <v/>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>~5% конверта (аналог холдинга 100 млрд)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>РАЛ</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>РосАгроЛизинг</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Оборудование (птичники, УПК, инкубатор, холод)</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>2340</v>
+      </c>
+      <c r="E7">
+        <f>D7/$B$3</f>
+        <v/>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>19,5% блока — как кролики 2 147,7 / 11 041,5</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ФРП</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Фонд развития промышленности</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <f>D8/$B$3</f>
+        <v/>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>ККЗ вне блока; корм с завода холдинга</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Банки</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Коммерческие банки</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>СМР, здания, инженерные сети</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>6287</v>
+      </c>
+      <c r="E9">
+        <f>D9/$B$3</f>
+        <v/>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>69,4% банковской доли (как СМР у кроликов)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Банки</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Коммерческие банки</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Solar 10 МВт·ч</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1180.8</v>
+      </c>
+      <c r="E10">
+        <f>D10/$B$3</f>
+        <v/>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>эталон кроликов tab#23</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Банки</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Коммерческие банки</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Комpost помёта 5 т/ч</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>36</v>
+      </c>
+      <c r="E11">
+        <f>D11/$B$3</f>
+        <v/>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>эталон кроликов tab#23</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Банки</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Коммерческие банки</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Проектирование, пусконаладка</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>27</v>
+      </c>
+      <c r="E12">
+        <f>D12/$B$3</f>
+        <v/>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>аналог строки «Проектирование» у кроликов</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Банки</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Коммерческие банки</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Родительское стадо, стартовый молодняк</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>463</v>
+      </c>
+      <c r="E13">
+        <f>D13/$B$3</f>
+        <v/>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>аналог «племенные» у кроликов</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Банки</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Коммерческие банки</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Оборотные средства</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>700</v>
+      </c>
+      <c r="E14">
+        <f>D14/$B$3</f>
+        <v/>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>как кролики (700 млн)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Банки</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Коммерческие банки</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Резерв + прочая инфраструктура</t>
+        </is>
+      </c>
+      <c r="D15">
+        <f>12000-SUM(D6:D14)</f>
+        <v/>
+      </c>
+      <c r="E15">
+        <f>D15/$B$3</f>
+        <v/>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>баланс до 12 000 (= CAPEX)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ИТОГО</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16">
+        <f>SUM(D6:D15)</f>
+        <v/>
+      </c>
+      <c r="E16">
+        <f>D16/$B$3</f>
+        <v/>
+      </c>
+      <c r="F16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="118" t="inlineStr">
+        <is>
+          <t>Примечание</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ККЗ и биогаз APK 20 МВт·ч — на уровне холдинга, не в CAPEX/OPEX блока птицы.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Детализация CAPEX — лист «CAPEX»; операционная модель — «Экономика», «NPV-IRR».</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -1244,201 +1719,200 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="58" t="inlineStr">
         <is>
           <t>МЕТОДОЛОГИЯ И ЭТАЛОН BASELINE (КРОЛИКИ)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="58" t="inlineStr">
         <is>
           <t>Параметр</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="58" t="inlineStr">
         <is>
           <t>Ед.</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="58" t="inlineStr">
         <is>
           <t>Значение</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="58" t="inlineStr">
         <is>
           <t>Источник / комментарий</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="58" t="inlineStr">
         <is>
           <t>Ставка дисконтирования (для NPV/IRR)</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="58" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="C19" t="n">
+      <c r="C19" s="58" t="n">
         <v>10</v>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="58" t="inlineStr">
         <is>
           <t>docs/1.ТЭО_МОЯ МЕЧТА.docx tab#7</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="58" t="inlineStr">
         <is>
           <t>CAPEX solar на блоке</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="58" t="inlineStr">
         <is>
           <t>МВт·ч / млн ₽</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="58" t="inlineStr">
         <is>
           <t>10 / 1180,8</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="58" t="inlineStr">
         <is>
           <t>tab#23; = кролики</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="58" t="inlineStr">
         <is>
           <t>CAPEX компost помёта</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="58" t="inlineStr">
         <is>
           <t>т/ч / млн ₽</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="58" t="inlineStr">
         <is>
           <t>5 / 36</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="58" t="inlineStr">
         <is>
           <t>tab#23; = кролики</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="58" t="inlineStr">
         <is>
           <t>Локальный biogaz+ГПU в блоке</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="58" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="58" t="inlineStr">
         <is>
           <t>как кролики; помёт → APK 20 МВт·ч</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="58" t="inlineStr">
         <is>
           <t>OPEX покупное электро</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="58" t="inlineStr">
         <is>
           <t>млн ₽/год</t>
         </is>
       </c>
-      <c r="C23" t="n">
+      <c r="C23" s="58" t="n">
         <v>0</v>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="58" t="inlineStr">
         <is>
           <t>у кроликов строки нет</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="58" t="inlineStr">
         <is>
           <t>Удобрение из органики</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="58" t="inlineStr">
         <is>
           <t>т/год × ₽/кг</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="58" t="inlineStr">
         <is>
           <t>43 800 × 12</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="58" t="inlineStr">
         <is>
           <t>tab#4,#205; сырьё — помёт птицы</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="58" t="inlineStr">
         <is>
           <t>ККЗ в CAPEX блока</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="58" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="58" t="inlineStr">
         <is>
           <t>корм с ККЗ холдинга ~28 000 ₽/т; у кроликов ККЗ 958,5 млн в docx</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="58" t="inlineStr">
         <is>
           <t>Горизонт finmodel</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="58" t="inlineStr">
         <is>
           <t>лет</t>
         </is>
       </c>
-      <c r="C26" t="n">
+      <c r="C26" s="58" t="n">
         <v>10</v>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="58" t="inlineStr">
         <is>
           <t>2026–2035, лист «Экономика»</t>
         </is>
@@ -1864,7 +2338,7 @@
         <v/>
       </c>
       <c r="F4" s="90">
-        <f>E4/Выручка!$E$12</f>
+        <f>E4/Выручка!$E$13</f>
         <v/>
       </c>
     </row>
@@ -1892,7 +2366,7 @@
         <v/>
       </c>
       <c r="F5" s="90">
-        <f>E5/Выручка!$E$12</f>
+        <f>E5/Выручка!$E$13</f>
         <v/>
       </c>
     </row>
@@ -1920,7 +2394,7 @@
         <v/>
       </c>
       <c r="F6" s="90">
-        <f>E6/Выручка!$E$12</f>
+        <f>E6/Выручка!$E$13</f>
         <v/>
       </c>
     </row>
@@ -1948,7 +2422,7 @@
         <v/>
       </c>
       <c r="F7" s="90">
-        <f>E7/Выручка!$E$12</f>
+        <f>E7/Выручка!$E$13</f>
         <v/>
       </c>
     </row>
@@ -1976,7 +2450,7 @@
         <v/>
       </c>
       <c r="F8" s="90">
-        <f>E8/Выручка!$E$12</f>
+        <f>E8/Выручка!$E$13</f>
         <v/>
       </c>
     </row>
@@ -2004,7 +2478,7 @@
         <v/>
       </c>
       <c r="F9" s="90">
-        <f>E9/Выручка!$E$12</f>
+        <f>E9/Выручка!$E$13</f>
         <v/>
       </c>
     </row>
@@ -2032,7 +2506,7 @@
         <v/>
       </c>
       <c r="F10" s="90">
-        <f>E10/Выручка!$E$12</f>
+        <f>E10/Выручка!$E$13</f>
         <v/>
       </c>
     </row>
@@ -2054,27 +2528,27 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="59">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="58" t="inlineStr">
         <is>
           <t>Удобрение из помёта (43 800 т/год × 12 ₽/кг, этalon кроликов tab#205)</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" s="58" t="n">
         <v>43800</v>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="58" t="inlineStr">
         <is>
           <t>т</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="58" t="n">
         <v>12</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="58">
         <f>B12*D12*1000/1000000</f>
         <v/>
       </c>
-      <c r="F12">
+      <c r="F12" s="58">
         <f>E12/Выручка!$E$13</f>
         <v/>
       </c>
@@ -2098,7 +2572,7 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="59">
-      <c r="E14">
+      <c r="E14" s="58">
         <f>(E4+E9+E10)/Выручка!$E$13</f>
         <v/>
       </c>
@@ -2110,7 +2584,7 @@
         </is>
       </c>
       <c r="E15" s="98">
-        <f>(E4+E9+E10)/Выручка!$E$12</f>
+        <f>(E4+E9+E10)/Выручка!$E$13</f>
         <v/>
       </c>
     </row>
@@ -2363,7 +2837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="48" customWidth="1" style="58" min="1" max="1"/>
@@ -2693,21 +3167,21 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="59">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="58" t="inlineStr">
         <is>
           <t>Установка компостирования помёта 5 т/ч (эталон кроликов)</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C17" s="58" t="n">
         <v>36</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D17" s="58" t="n">
         <v>36</v>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="58" t="inlineStr">
         <is>
           <t>Общая инфраструктура</t>
         </is>
@@ -2723,7 +3197,7 @@
         <v>1</v>
       </c>
       <c r="C18" s="103" t="n">
-        <v>1000</v>
+        <v>750</v>
       </c>
       <c r="D18" s="82">
         <f>B17*C17</f>
@@ -2767,7 +3241,7 @@
         <v>1</v>
       </c>
       <c r="C20" s="103" t="n">
-        <v>250</v>
+        <v>183</v>
       </c>
       <c r="D20" s="82">
         <f>B19*C19</f>
@@ -2811,7 +3285,7 @@
         <v>1</v>
       </c>
       <c r="C22" s="103" t="n">
-        <v>450</v>
+        <v>250</v>
       </c>
       <c r="D22" s="82">
         <f>B21*C21</f>
@@ -2877,7 +3351,7 @@
         <v>1</v>
       </c>
       <c r="C25" s="103" t="n">
-        <v>400</v>
+        <v>33</v>
       </c>
       <c r="D25" s="82">
         <f>12000-SUM(D4:D24)</f>
@@ -3214,7 +3688,7 @@
         </is>
       </c>
       <c r="B4" s="109">
-        <f>CAPEX!$D$25</f>
+        <f>CAPEX!$D$26</f>
         <v/>
       </c>
     </row>
@@ -3604,4 +4078,840 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" style="59" min="1" max="1"/>
+    <col width="14" customWidth="1" style="59" min="2" max="2"/>
+    <col width="14" customWidth="1" style="59" min="3" max="3"/>
+    <col width="14" customWidth="1" style="59" min="4" max="4"/>
+    <col width="14" customWidth="1" style="59" min="5" max="5"/>
+    <col width="14" customWidth="1" style="59" min="6" max="6"/>
+    <col width="14" customWidth="1" style="59" min="7" max="7"/>
+    <col width="14" customWidth="1" style="59" min="8" max="8"/>
+    <col width="14" customWidth="1" style="59" min="9" max="9"/>
+    <col width="14" customWidth="1" style="59" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="116" t="inlineStr">
+        <is>
+          <t>NPV / IRR — DCF @ 10% (эталон кроликов, tab#7 docx)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Горизонт 2026–2035 · без долга · FCF = ЧП + амортизация · CAPEX в 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ставка дисконтирования</t>
+        </is>
+      </c>
+      <c r="B3">
+        <f>Допущения!C19</f>
+        <v/>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="117" t="inlineStr">
+        <is>
+          <t>Год</t>
+        </is>
+      </c>
+      <c r="B5" s="117" t="inlineStr">
+        <is>
+          <t>Загрузка</t>
+        </is>
+      </c>
+      <c r="C5" s="117" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="D5" s="117" t="inlineStr">
+        <is>
+          <t>Аморт.</t>
+        </is>
+      </c>
+      <c r="E5" s="117" t="inlineStr">
+        <is>
+          <t>Прибыль до налога</t>
+        </is>
+      </c>
+      <c r="F5" s="117" t="inlineStr">
+        <is>
+          <t>Налог ЕСХН 6%</t>
+        </is>
+      </c>
+      <c r="G5" s="117" t="inlineStr">
+        <is>
+          <t>Чистая прибыль</t>
+        </is>
+      </c>
+      <c r="H5" s="117" t="inlineStr">
+        <is>
+          <t>FCF</t>
+        </is>
+      </c>
+      <c r="I5" s="117" t="inlineStr">
+        <is>
+          <t>DF @ 10%</t>
+        </is>
+      </c>
+      <c r="J5" s="117" t="inlineStr">
+        <is>
+          <t>PV FCF</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B6">
+        <f>Экономика!B22</f>
+        <v/>
+      </c>
+      <c r="C6">
+        <f>Экономика!B24</f>
+        <v/>
+      </c>
+      <c r="D6">
+        <f>IF(B6&gt;0,Экономика!$B$9*B6,0)</f>
+        <v/>
+      </c>
+      <c r="E6">
+        <f>C6-D6</f>
+        <v/>
+      </c>
+      <c r="F6">
+        <f>MAX(E6*0.06,0)</f>
+        <v/>
+      </c>
+      <c r="G6">
+        <f>E6-F6</f>
+        <v/>
+      </c>
+      <c r="H6">
+        <f>G6+D6-Экономика!$B$4</f>
+        <v/>
+      </c>
+      <c r="I6">
+        <f>1/(1+$B$3/100)^(6-5)</f>
+        <v/>
+      </c>
+      <c r="J6">
+        <f>H6*I6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B7">
+        <f>Экономика!C22</f>
+        <v/>
+      </c>
+      <c r="C7">
+        <f>Экономика!C24</f>
+        <v/>
+      </c>
+      <c r="D7">
+        <f>IF(B7&gt;0,Экономика!$B$9*B7,0)</f>
+        <v/>
+      </c>
+      <c r="E7">
+        <f>C7-D7</f>
+        <v/>
+      </c>
+      <c r="F7">
+        <f>MAX(E7*0.06,0)</f>
+        <v/>
+      </c>
+      <c r="G7">
+        <f>E7-F7</f>
+        <v/>
+      </c>
+      <c r="H7">
+        <f>G7+D7</f>
+        <v/>
+      </c>
+      <c r="I7">
+        <f>1/(1+$B$3/100)^(7-5)</f>
+        <v/>
+      </c>
+      <c r="J7">
+        <f>H7*I7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2028</v>
+      </c>
+      <c r="B8">
+        <f>Экономика!D22</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>Экономика!D24</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>IF(B8&gt;0,Экономика!$B$9*B8,0)</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>C8-D8</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>MAX(E8*0.06,0)</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>E8-F8</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>G8+D8</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>1/(1+$B$3/100)^(8-5)</f>
+        <v/>
+      </c>
+      <c r="J8">
+        <f>H8*I8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2029</v>
+      </c>
+      <c r="B9">
+        <f>Экономика!E22</f>
+        <v/>
+      </c>
+      <c r="C9">
+        <f>Экономика!E24</f>
+        <v/>
+      </c>
+      <c r="D9">
+        <f>IF(B9&gt;0,Экономика!$B$9*B9,0)</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>C9-D9</f>
+        <v/>
+      </c>
+      <c r="F9">
+        <f>MAX(E9*0.06,0)</f>
+        <v/>
+      </c>
+      <c r="G9">
+        <f>E9-F9</f>
+        <v/>
+      </c>
+      <c r="H9">
+        <f>G9+D9</f>
+        <v/>
+      </c>
+      <c r="I9">
+        <f>1/(1+$B$3/100)^(9-5)</f>
+        <v/>
+      </c>
+      <c r="J9">
+        <f>H9*I9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2030</v>
+      </c>
+      <c r="B10">
+        <f>Экономика!F22</f>
+        <v/>
+      </c>
+      <c r="C10">
+        <f>Экономика!F24</f>
+        <v/>
+      </c>
+      <c r="D10">
+        <f>IF(B10&gt;0,Экономика!$B$9*B10,0)</f>
+        <v/>
+      </c>
+      <c r="E10">
+        <f>C10-D10</f>
+        <v/>
+      </c>
+      <c r="F10">
+        <f>MAX(E10*0.06,0)</f>
+        <v/>
+      </c>
+      <c r="G10">
+        <f>E10-F10</f>
+        <v/>
+      </c>
+      <c r="H10">
+        <f>G10+D10</f>
+        <v/>
+      </c>
+      <c r="I10">
+        <f>1/(1+$B$3/100)^(10-5)</f>
+        <v/>
+      </c>
+      <c r="J10">
+        <f>H10*I10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2031</v>
+      </c>
+      <c r="B11">
+        <f>Экономика!G22</f>
+        <v/>
+      </c>
+      <c r="C11">
+        <f>Экономика!G24</f>
+        <v/>
+      </c>
+      <c r="D11">
+        <f>IF(B11&gt;0,Экономика!$B$9*B11,0)</f>
+        <v/>
+      </c>
+      <c r="E11">
+        <f>C11-D11</f>
+        <v/>
+      </c>
+      <c r="F11">
+        <f>MAX(E11*0.06,0)</f>
+        <v/>
+      </c>
+      <c r="G11">
+        <f>E11-F11</f>
+        <v/>
+      </c>
+      <c r="H11">
+        <f>G11+D11</f>
+        <v/>
+      </c>
+      <c r="I11">
+        <f>1/(1+$B$3/100)^(11-5)</f>
+        <v/>
+      </c>
+      <c r="J11">
+        <f>H11*I11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2032</v>
+      </c>
+      <c r="B12">
+        <f>Экономика!H22</f>
+        <v/>
+      </c>
+      <c r="C12">
+        <f>Экономика!H24</f>
+        <v/>
+      </c>
+      <c r="D12">
+        <f>IF(B12&gt;0,Экономика!$B$9*B12,0)</f>
+        <v/>
+      </c>
+      <c r="E12">
+        <f>C12-D12</f>
+        <v/>
+      </c>
+      <c r="F12">
+        <f>MAX(E12*0.06,0)</f>
+        <v/>
+      </c>
+      <c r="G12">
+        <f>E12-F12</f>
+        <v/>
+      </c>
+      <c r="H12">
+        <f>G12+D12</f>
+        <v/>
+      </c>
+      <c r="I12">
+        <f>1/(1+$B$3/100)^(12-5)</f>
+        <v/>
+      </c>
+      <c r="J12">
+        <f>H12*I12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2033</v>
+      </c>
+      <c r="B13">
+        <f>Экономика!I22</f>
+        <v/>
+      </c>
+      <c r="C13">
+        <f>Экономика!I24</f>
+        <v/>
+      </c>
+      <c r="D13">
+        <f>IF(B13&gt;0,Экономика!$B$9*B13,0)</f>
+        <v/>
+      </c>
+      <c r="E13">
+        <f>C13-D13</f>
+        <v/>
+      </c>
+      <c r="F13">
+        <f>MAX(E13*0.06,0)</f>
+        <v/>
+      </c>
+      <c r="G13">
+        <f>E13-F13</f>
+        <v/>
+      </c>
+      <c r="H13">
+        <f>G13+D13</f>
+        <v/>
+      </c>
+      <c r="I13">
+        <f>1/(1+$B$3/100)^(13-5)</f>
+        <v/>
+      </c>
+      <c r="J13">
+        <f>H13*I13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2034</v>
+      </c>
+      <c r="B14">
+        <f>Экономика!J22</f>
+        <v/>
+      </c>
+      <c r="C14">
+        <f>Экономика!J24</f>
+        <v/>
+      </c>
+      <c r="D14">
+        <f>IF(B14&gt;0,Экономика!$B$9*B14,0)</f>
+        <v/>
+      </c>
+      <c r="E14">
+        <f>C14-D14</f>
+        <v/>
+      </c>
+      <c r="F14">
+        <f>MAX(E14*0.06,0)</f>
+        <v/>
+      </c>
+      <c r="G14">
+        <f>E14-F14</f>
+        <v/>
+      </c>
+      <c r="H14">
+        <f>G14+D14</f>
+        <v/>
+      </c>
+      <c r="I14">
+        <f>1/(1+$B$3/100)^(14-5)</f>
+        <v/>
+      </c>
+      <c r="J14">
+        <f>H14*I14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>2035</v>
+      </c>
+      <c r="B15">
+        <f>Экономика!K22</f>
+        <v/>
+      </c>
+      <c r="C15">
+        <f>Экономика!K24</f>
+        <v/>
+      </c>
+      <c r="D15">
+        <f>IF(B15&gt;0,Экономика!$B$9*B15,0)</f>
+        <v/>
+      </c>
+      <c r="E15">
+        <f>C15-D15</f>
+        <v/>
+      </c>
+      <c r="F15">
+        <f>MAX(E15*0.06,0)</f>
+        <v/>
+      </c>
+      <c r="G15">
+        <f>E15-F15</f>
+        <v/>
+      </c>
+      <c r="H15">
+        <f>G15+D15</f>
+        <v/>
+      </c>
+      <c r="I15">
+        <f>1/(1+$B$3/100)^(15-5)</f>
+        <v/>
+      </c>
+      <c r="J15">
+        <f>H15*I15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2036</v>
+      </c>
+      <c r="B16">
+        <f>1</f>
+        <v/>
+      </c>
+      <c r="C16">
+        <f>Экономика!$B$7</f>
+        <v/>
+      </c>
+      <c r="D16">
+        <f>IF(B16&gt;0,Экономика!$B$9*B16,0)</f>
+        <v/>
+      </c>
+      <c r="E16">
+        <f>C16-D16</f>
+        <v/>
+      </c>
+      <c r="F16">
+        <f>MAX(E16*0.06,0)</f>
+        <v/>
+      </c>
+      <c r="G16">
+        <f>E16-F16</f>
+        <v/>
+      </c>
+      <c r="H16">
+        <f>G16+D16</f>
+        <v/>
+      </c>
+      <c r="I16">
+        <f>1/(1+$B$3/100)^(16-5)</f>
+        <v/>
+      </c>
+      <c r="J16">
+        <f>H16*I16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>2037</v>
+      </c>
+      <c r="B17">
+        <f>1</f>
+        <v/>
+      </c>
+      <c r="C17">
+        <f>Экономика!$B$7</f>
+        <v/>
+      </c>
+      <c r="D17">
+        <f>IF(B17&gt;0,Экономика!$B$9*B17,0)</f>
+        <v/>
+      </c>
+      <c r="E17">
+        <f>C17-D17</f>
+        <v/>
+      </c>
+      <c r="F17">
+        <f>MAX(E17*0.06,0)</f>
+        <v/>
+      </c>
+      <c r="G17">
+        <f>E17-F17</f>
+        <v/>
+      </c>
+      <c r="H17">
+        <f>G17+D17</f>
+        <v/>
+      </c>
+      <c r="I17">
+        <f>1/(1+$B$3/100)^(17-5)</f>
+        <v/>
+      </c>
+      <c r="J17">
+        <f>H17*I17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>2038</v>
+      </c>
+      <c r="B18">
+        <f>1</f>
+        <v/>
+      </c>
+      <c r="C18">
+        <f>Экономика!$B$7</f>
+        <v/>
+      </c>
+      <c r="D18">
+        <f>IF(B18&gt;0,Экономика!$B$9*B18,0)</f>
+        <v/>
+      </c>
+      <c r="E18">
+        <f>C18-D18</f>
+        <v/>
+      </c>
+      <c r="F18">
+        <f>MAX(E18*0.06,0)</f>
+        <v/>
+      </c>
+      <c r="G18">
+        <f>E18-F18</f>
+        <v/>
+      </c>
+      <c r="H18">
+        <f>G18+D18</f>
+        <v/>
+      </c>
+      <c r="I18">
+        <f>1/(1+$B$3/100)^(18-5)</f>
+        <v/>
+      </c>
+      <c r="J18">
+        <f>H18*I18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>2039</v>
+      </c>
+      <c r="B19">
+        <f>1</f>
+        <v/>
+      </c>
+      <c r="C19">
+        <f>Экономика!$B$7</f>
+        <v/>
+      </c>
+      <c r="D19">
+        <f>IF(B19&gt;0,Экономика!$B$9*B19,0)</f>
+        <v/>
+      </c>
+      <c r="E19">
+        <f>C19-D19</f>
+        <v/>
+      </c>
+      <c r="F19">
+        <f>MAX(E19*0.06,0)</f>
+        <v/>
+      </c>
+      <c r="G19">
+        <f>E19-F19</f>
+        <v/>
+      </c>
+      <c r="H19">
+        <f>G19+D19</f>
+        <v/>
+      </c>
+      <c r="I19">
+        <f>1/(1+$B$3/100)^(19-5)</f>
+        <v/>
+      </c>
+      <c r="J19">
+        <f>H19*I19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>2040</v>
+      </c>
+      <c r="B20">
+        <f>1</f>
+        <v/>
+      </c>
+      <c r="C20">
+        <f>Экономика!$B$7</f>
+        <v/>
+      </c>
+      <c r="D20">
+        <f>IF(B20&gt;0,Экономика!$B$9*B20,0)</f>
+        <v/>
+      </c>
+      <c r="E20">
+        <f>C20-D20</f>
+        <v/>
+      </c>
+      <c r="F20">
+        <f>MAX(E20*0.06,0)</f>
+        <v/>
+      </c>
+      <c r="G20">
+        <f>E20-F20</f>
+        <v/>
+      </c>
+      <c r="H20">
+        <f>G20+D20</f>
+        <v/>
+      </c>
+      <c r="I20">
+        <f>1/(1+$B$3/100)^(20-5)</f>
+        <v/>
+      </c>
+      <c r="J20">
+        <f>H20*I20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>2041</v>
+      </c>
+      <c r="B21">
+        <f>1</f>
+        <v/>
+      </c>
+      <c r="C21">
+        <f>Экономика!$B$7</f>
+        <v/>
+      </c>
+      <c r="D21">
+        <f>IF(B21&gt;0,Экономика!$B$9*B21,0)</f>
+        <v/>
+      </c>
+      <c r="E21">
+        <f>C21-D21</f>
+        <v/>
+      </c>
+      <c r="F21">
+        <f>MAX(E21*0.06,0)</f>
+        <v/>
+      </c>
+      <c r="G21">
+        <f>E21-F21</f>
+        <v/>
+      </c>
+      <c r="H21">
+        <f>G21+D21</f>
+        <v/>
+      </c>
+      <c r="I21">
+        <f>1/(1+$B$3/100)^(21-5)</f>
+        <v/>
+      </c>
+      <c r="J21">
+        <f>H21*I21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="118" t="inlineStr">
+        <is>
+          <t>NPV @ 10%, млн ₽</t>
+        </is>
+      </c>
+      <c r="B22">
+        <f>SUM(J6:J21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="118" t="inlineStr">
+        <is>
+          <t>IRR, %</t>
+        </is>
+      </c>
+      <c r="B23">
+        <f>IRR(H6:H21)*100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="118" t="inlineStr">
+        <is>
+          <t>PI (NPV/CAPEX + 1)</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>B22/Экономика!B4+1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Сравнение с кроликами (docx tab#7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Кролики NPV @ 10%</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>2779.5</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Кролики IRR</t>
+        </is>
+      </c>
+      <c r="B28" s="119" t="n">
+        <v>0.1519</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Горизонт DCF</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>16 лет (2026–2041)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add APK 100 bln integration slide for poultry 12 bln block
- appendix/apk-100bln-integration.md: unified CAPEX/financing/infra slide
- finmodel xlsx sheet APK-100 linked to Financing sheet
- land-budget: 250k ha Zaporozhye base, cadastre pending
- Update poultry-teo.yaml and financing-structure.md

Co-authored-by: Demid369 <Demid369@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/teo-poultry/_incoming/finmodel-pticekompleks-12-mlrd.xlsx
+++ b/docs/teo-poultry/_incoming/finmodel-pticekompleks-12-mlrd.xlsx
@@ -17,6 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Экономика" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPV-IRR" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Финансирование" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="APK-100" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -1074,7 +1075,7 @@
     <row r="24">
       <c r="A24" s="58" t="inlineStr">
         <is>
-          <t>Подробности — листы: Продукция, Выручка, Корма, CAPEX, OPEX, Экономика, NPV-IRR, Финансирование, Допущения.</t>
+          <t>Подробности — листы: … CAPEX, OPEX, Экономика, NPV-IRR, Финансирование, APK-100, Допущения.</t>
         </is>
       </c>
     </row>
@@ -1112,7 +1113,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Шаблон: docs/1.2-слайд Фин модель.xlsx (ФНБ / РАЛ / ФРП / банки) · блок птицы отдельно от APK 100 млрд</t>
+          <t>Шаблон: docs/1.2-слайд Фин модель.xlsx · встройка в 100 млрд: лист «APK-100»</t>
         </is>
       </c>
     </row>
@@ -1486,6 +1487,379 @@
       <c r="A19" t="inlineStr">
         <is>
           <t>Детализация CAPEX — лист «CAPEX»; операционная модель — «Экономика», «NPV-IRR».</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="59" min="1" max="1"/>
+    <col width="42" customWidth="1" style="59" min="2" max="2"/>
+    <col width="18" customWidth="1" style="59" min="3" max="3"/>
+    <col width="18" customWidth="1" style="59" min="4" max="4"/>
+    <col width="18" customWidth="1" style="59" min="5" max="5"/>
+    <col width="18" customWidth="1" style="59" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="116" t="inlineStr">
+        <is>
+          <t>ВСТРОЙКА 12 млрд ПТИЦЫ В КОНТУР APK 100 млрд (Приложение 3Б)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Baseline: docs/1.2-слайд Фин модель.xlsx · блок птицы: finmodel · apk-100bln-integration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Земля птицы: APK 250 000 га, Запорожская обл. · слот 400 га · кадастр позже</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="117" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B5" s="117" t="inlineStr">
+        <is>
+          <t>Блок</t>
+        </is>
+      </c>
+      <c r="C5" s="117" t="inlineStr">
+        <is>
+          <t>Baseline (кролики), млн ₽</t>
+        </is>
+      </c>
+      <c r="D5" s="117" t="inlineStr">
+        <is>
+          <t>С птицей, млн ₽</t>
+        </is>
+      </c>
+      <c r="E5" s="117" t="inlineStr">
+        <is>
+          <t>Δ, млн ₽</t>
+        </is>
+      </c>
+      <c r="F5" s="117" t="inlineStr">
+        <is>
+          <t>Доля в 100,9 млрд</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Птицеводческий комплекс «Нова-Агро» (слот кроликов)</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>11041.5</v>
+      </c>
+      <c r="D6" t="n">
+        <v>12000</v>
+      </c>
+      <c r="E6">
+        <f>D6-C6</f>
+        <v/>
+      </c>
+      <c r="F6">
+        <f>D6/$D$11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Тепличный комплекс</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>34500</v>
+      </c>
+      <c r="D7" t="n">
+        <v>34500</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <f>D7/$D$11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Животноводческая ферма (КРС/МРС)</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>27458.5</v>
+      </c>
+      <c r="D8" t="n">
+        <v>27458.5</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <f>D8/$D$11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Рыбоводство (белуга)</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>9000</v>
+      </c>
+      <c r="D9" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <f>D9/$D$11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Масложировой комбинат</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>18000</v>
+      </c>
+      <c r="D10" t="n">
+        <v>18000</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <f>D10/$D$11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="118" t="n"/>
+      <c r="B11" s="118" t="inlineStr">
+        <is>
+          <t>ИТОГО APK</t>
+        </is>
+      </c>
+      <c r="C11" s="118">
+        <f>SUM(C6:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="118">
+        <f>SUM(D6:D10)</f>
+        <v/>
+      </c>
+      <c r="E11" s="118">
+        <f>D11-C11</f>
+        <v/>
+      </c>
+      <c r="F11" s="118" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="118" t="inlineStr">
+        <is>
+          <t>Источники финансирования блока 1 (12 000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="117" t="inlineStr">
+        <is>
+          <t>Источник</t>
+        </is>
+      </c>
+      <c r="B14" s="117" t="inlineStr">
+        <is>
+          <t>млн ₽</t>
+        </is>
+      </c>
+      <c r="C14" s="117" t="inlineStr">
+        <is>
+          <t>Доля блока</t>
+        </is>
+      </c>
+      <c r="D14" s="117" t="inlineStr">
+        <is>
+          <t>Ссылка</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ФНБ</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>Финансирование!D6</f>
+        <v/>
+      </c>
+      <c r="C15">
+        <f>Финансирование!E6</f>
+        <v/>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>лист Финансирование</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>РАЛ</t>
+        </is>
+      </c>
+      <c r="B16">
+        <f>Финансирование!D7</f>
+        <v/>
+      </c>
+      <c r="C16">
+        <f>Финансирование!E7</f>
+        <v/>
+      </c>
+      <c r="D16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ФРП</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>Финансирование!D8</f>
+        <v/>
+      </c>
+      <c r="C17">
+        <f>Финансирование!E8</f>
+        <v/>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>ККЗ вне блока</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Банки</t>
+        </is>
+      </c>
+      <c r="B18">
+        <f>SUM(Финансирование!D9:D15)</f>
+        <v/>
+      </c>
+      <c r="C18">
+        <f>B18/12000</f>
+        <v/>
+      </c>
+      <c r="D18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Итого блок 1</t>
+        </is>
+      </c>
+      <c r="B19">
+        <f>SUM(B15:B18)</f>
+        <v/>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Общая инфра APK (без изменений)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ККЗ 300 тыс. т/год</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>корм птицы ~22% мощности</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Биogaz APK 20 МВт·ч</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>помёт птицы → установка холдинга</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Solar 50 МВт·ч</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>10 МВт·ч на блоке птицы (CAPEX 12 млрд)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Calculate sensitivity, export hypotheses, APK 100 bln scenarios
- scripts/calc-poultry-scenarios.py: 9 sensitivity cases, 4 export, 3 APK-100
- xlsx sheets Чувствительность and Экспорт
- appendix/sensitivity-and-scenarios.md, calculated-scenarios.json
- T09 SWOT and competitor table filled

Co-authored-by: Demid369 <Demid369@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/teo-poultry/_incoming/finmodel-pticekompleks-12-mlrd.xlsx
+++ b/docs/teo-poultry/_incoming/finmodel-pticekompleks-12-mlrd.xlsx
@@ -18,6 +18,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPV-IRR" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Финансирование" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="APK-100" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Чувствительность" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Экспорт" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -244,7 +246,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="120">
+  <cellXfs count="122">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -597,6 +599,8 @@
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1111,22 +1115,22 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="58" t="inlineStr">
         <is>
           <t>Шаблон: docs/1.2-слайд Фин модель.xlsx · встройка в 100 млрд: лист «APK-100»</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="58" t="inlineStr">
         <is>
           <t>Сумма инвестиций</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="58" t="n">
         <v>12000</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="58" t="inlineStr">
         <is>
           <t>млн ₽</t>
         </is>
@@ -1161,313 +1165,313 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="58" t="inlineStr">
         <is>
           <t>ФНБ</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="58" t="inlineStr">
         <is>
           <t>Фонд национального благосостояния</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="58" t="inlineStr">
         <is>
           <t>Долевое участие в проекте</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="58" t="n">
         <v>600</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="58">
         <f>D6/$B$3</f>
         <v/>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="58" t="inlineStr">
         <is>
           <t>~5% конверта (аналог холдинга 100 млрд)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="58" t="inlineStr">
         <is>
           <t>РАЛ</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="58" t="inlineStr">
         <is>
           <t>РосАгроЛизинг</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="58" t="inlineStr">
         <is>
           <t>Оборудование (птичники, УПК, инкубатор, холод)</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="58" t="n">
         <v>2340</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="58">
         <f>D7/$B$3</f>
         <v/>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="58" t="inlineStr">
         <is>
           <t>19,5% блока — как кролики 2 147,7 / 11 041,5</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="58" t="inlineStr">
         <is>
           <t>ФРП</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="58" t="inlineStr">
         <is>
           <t>Фонд развития промышленности</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="58" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="58" t="n">
         <v>0</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="58">
         <f>D8/$B$3</f>
         <v/>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="58" t="inlineStr">
         <is>
           <t>ККЗ вне блока; корм с завода холдинга</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="58" t="inlineStr">
         <is>
           <t>Банки</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="58" t="inlineStr">
         <is>
           <t>Коммерческие банки</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="58" t="inlineStr">
         <is>
           <t>СМР, здания, инженерные сети</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="58" t="n">
         <v>6287</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="58">
         <f>D9/$B$3</f>
         <v/>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="58" t="inlineStr">
         <is>
           <t>69,4% банковской доли (как СМР у кроликов)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="58" t="inlineStr">
         <is>
           <t>Банки</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="58" t="inlineStr">
         <is>
           <t>Коммерческие банки</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="58" t="inlineStr">
         <is>
           <t>Solar 10 МВт·ч</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="58" t="n">
         <v>1180.8</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="58">
         <f>D10/$B$3</f>
         <v/>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="58" t="inlineStr">
         <is>
           <t>эталон кроликов tab#23</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="58" t="inlineStr">
         <is>
           <t>Банки</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="58" t="inlineStr">
         <is>
           <t>Коммерческие банки</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="58" t="inlineStr">
         <is>
           <t>Комpost помёта 5 т/ч</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="58" t="n">
         <v>36</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="58">
         <f>D11/$B$3</f>
         <v/>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="58" t="inlineStr">
         <is>
           <t>эталон кроликов tab#23</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="58" t="inlineStr">
         <is>
           <t>Банки</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="58" t="inlineStr">
         <is>
           <t>Коммерческие банки</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="58" t="inlineStr">
         <is>
           <t>Проектирование, пусконаладка</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="58" t="n">
         <v>27</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="58">
         <f>D12/$B$3</f>
         <v/>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="58" t="inlineStr">
         <is>
           <t>аналог строки «Проектирование» у кроликов</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="58" t="inlineStr">
         <is>
           <t>Банки</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="58" t="inlineStr">
         <is>
           <t>Коммерческие банки</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="58" t="inlineStr">
         <is>
           <t>Родительское стадо, стартовый молодняк</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" s="58" t="n">
         <v>463</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="58">
         <f>D13/$B$3</f>
         <v/>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="58" t="inlineStr">
         <is>
           <t>аналог «племенные» у кроликов</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="58" t="inlineStr">
         <is>
           <t>Банки</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="58" t="inlineStr">
         <is>
           <t>Коммерческие банки</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="58" t="inlineStr">
         <is>
           <t>Оборотные средства</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" s="58" t="n">
         <v>700</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="58">
         <f>D14/$B$3</f>
         <v/>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="58" t="inlineStr">
         <is>
           <t>как кролики (700 млн)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="58" t="inlineStr">
         <is>
           <t>Банки</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="58" t="inlineStr">
         <is>
           <t>Коммерческие банки</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="58" t="inlineStr">
         <is>
           <t>Резерв + прочая инфраструктура</t>
         </is>
       </c>
-      <c r="D15">
+      <c r="D15" s="58">
         <f>12000-SUM(D6:D14)</f>
         <v/>
       </c>
-      <c r="E15">
+      <c r="E15" s="58">
         <f>D15/$B$3</f>
         <v/>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" s="58" t="inlineStr">
         <is>
           <t>баланс до 12 000 (= CAPEX)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr">
+      <c r="A16" s="58" t="inlineStr"/>
+      <c r="B16" s="58" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16">
+      <c r="C16" s="58" t="inlineStr"/>
+      <c r="D16" s="58">
         <f>SUM(D6:D15)</f>
         <v/>
       </c>
-      <c r="E16">
+      <c r="E16" s="58">
         <f>D16/$B$3</f>
         <v/>
       </c>
-      <c r="F16" t="inlineStr"/>
+      <c r="F16" s="58" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="118" t="inlineStr">
@@ -1477,14 +1481,14 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="58" t="inlineStr">
         <is>
           <t>ККЗ и биогаз APK 20 МВт·ч — на уровне холдинга, не в CAPEX/OPEX блока птицы.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="58" t="inlineStr">
         <is>
           <t>Детализация CAPEX — лист «CAPEX»; операционная модель — «Экономика», «NPV-IRR».</t>
         </is>
@@ -1501,7 +1505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="59" min="1" max="1"/>
@@ -1520,14 +1524,14 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="58" t="inlineStr">
         <is>
           <t>Baseline: docs/1.2-слайд Фин модель.xlsx · блок птицы: finmodel · apk-100bln-integration.md</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="58" t="inlineStr">
         <is>
           <t>Земля птицы: APK 250 000 га, Запорожская обл. · слот 400 га · кадастр позже</t>
         </is>
@@ -1566,117 +1570,117 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="58" t="inlineStr">
         <is>
           <t>Птицеводческий комплекс «Нова-Агро» (слот кроликов)</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="58" t="n">
         <v>11041.5</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="58" t="n">
         <v>12000</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="58">
         <f>D6-C6</f>
         <v/>
       </c>
-      <c r="F6">
+      <c r="F6" s="58">
         <f>D6/$D$11</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="58" t="n">
         <v>2</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="58" t="inlineStr">
         <is>
           <t>Тепличный комплекс</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="58" t="n">
         <v>34500</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="58" t="n">
         <v>34500</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="58" t="n">
         <v>0</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="58">
         <f>D7/$D$11</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="58" t="n">
         <v>3</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="58" t="inlineStr">
         <is>
           <t>Животноводческая ферма (КРС/МРС)</t>
         </is>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" s="58" t="n">
         <v>27458.5</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="58" t="n">
         <v>27458.5</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="58" t="n">
         <v>0</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="58">
         <f>D8/$D$11</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="58" t="n">
         <v>4</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="58" t="inlineStr">
         <is>
           <t>Рыбоводство (белуга)</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" s="58" t="n">
         <v>9000</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="58" t="n">
         <v>9000</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="58" t="n">
         <v>0</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="58">
         <f>D9/$D$11</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="58" t="n">
         <v>5</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="58" t="inlineStr">
         <is>
           <t>Масложировой комбинат</t>
         </is>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" s="58" t="n">
         <v>18000</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="58" t="n">
         <v>18000</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="58" t="n">
         <v>0</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="58">
         <f>D10/$D$11</f>
         <v/>
       </c>
@@ -1734,132 +1738,736 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="58" t="inlineStr">
         <is>
           <t>ФНБ</t>
         </is>
       </c>
-      <c r="B15">
+      <c r="B15" s="58">
         <f>Финансирование!D6</f>
         <v/>
       </c>
-      <c r="C15">
+      <c r="C15" s="58">
         <f>Финансирование!E6</f>
         <v/>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="58" t="inlineStr">
         <is>
           <t>лист Финансирование</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="58" t="inlineStr">
         <is>
           <t>РАЛ</t>
         </is>
       </c>
-      <c r="B16">
+      <c r="B16" s="58">
         <f>Финансирование!D7</f>
         <v/>
       </c>
-      <c r="C16">
+      <c r="C16" s="58">
         <f>Финансирование!E7</f>
         <v/>
       </c>
-      <c r="D16" t="inlineStr"/>
+      <c r="D16" s="58" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="58" t="inlineStr">
         <is>
           <t>ФРП</t>
         </is>
       </c>
-      <c r="B17">
+      <c r="B17" s="58">
         <f>Финансирование!D8</f>
         <v/>
       </c>
-      <c r="C17">
+      <c r="C17" s="58">
         <f>Финансирование!E8</f>
         <v/>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="58" t="inlineStr">
         <is>
           <t>ККЗ вне блока</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="58" t="inlineStr">
         <is>
           <t>Банки</t>
         </is>
       </c>
-      <c r="B18">
+      <c r="B18" s="58">
         <f>SUM(Финансирование!D9:D15)</f>
         <v/>
       </c>
-      <c r="C18">
+      <c r="C18" s="58">
         <f>B18/12000</f>
         <v/>
       </c>
-      <c r="D18" t="inlineStr"/>
+      <c r="D18" s="58" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="58" t="inlineStr">
         <is>
           <t>Итого блок 1</t>
         </is>
       </c>
-      <c r="B19">
+      <c r="B19" s="58">
         <f>SUM(B15:B18)</f>
         <v/>
       </c>
-      <c r="C19" t="n">
+      <c r="C19" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="D19" t="inlineStr"/>
+      <c r="D19" s="58" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="58" t="inlineStr">
         <is>
           <t>Общая инфра APK (без изменений)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="58" t="inlineStr">
         <is>
           <t>ККЗ 300 тыс. т/год</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="58" t="inlineStr">
         <is>
           <t>корм птицы ~22% мощности</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="58" t="inlineStr">
         <is>
           <t>Биogaz APK 20 МВт·ч</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="58" t="inlineStr">
         <is>
           <t>помёт птицы → установка холдинга</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="58" t="inlineStr">
         <is>
           <t>Solar 50 МВт·ч</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="58" t="inlineStr">
         <is>
           <t>10 МВт·ч на блоке птицы (CAPEX 12 млрд)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="118" t="inlineStr">
+        <is>
+          <t>Сценарий C: итог ровно 100 000</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="58" t="inlineStr">
+        <is>
+          <t>Птица / кролики (блок 1)</t>
+        </is>
+      </c>
+      <c r="B27" s="58" t="n">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="58" t="inlineStr">
+        <is>
+          <t>Теплицы</t>
+        </is>
+      </c>
+      <c r="B28" s="58" t="n">
+        <v>34128.3</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="58" t="inlineStr">
+        <is>
+          <t>Животноводство</t>
+        </is>
+      </c>
+      <c r="B29" s="58" t="n">
+        <v>27162.6</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="58" t="inlineStr">
+        <is>
+          <t>Рыба</t>
+        </is>
+      </c>
+      <c r="B30" s="58" t="n">
+        <v>8903</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="58" t="inlineStr">
+        <is>
+          <t>Масложир</t>
+        </is>
+      </c>
+      <c r="B31" s="58" t="n">
+        <v>17806.1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="58" t="inlineStr">
+        <is>
+          <t>ИТОГО</t>
+        </is>
+      </c>
+      <c r="B32" s="58" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="116" t="inlineStr">
+        <is>
+          <t>АНАЛИЗ ЧУВСТВИТЕЛЬНОСТИ — полная мощность</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>NPV/IRR: DCF 16 лет @10%, как лист NPV-IRR · расчёт scripts/calc-poultry-scenarios.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="120" t="inlineStr">
+        <is>
+          <t>Сценарий</t>
+        </is>
+      </c>
+      <c r="B4" s="120" t="inlineStr">
+        <is>
+          <t>Выручка</t>
+        </is>
+      </c>
+      <c r="C4" s="120" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="D4" s="120" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="E4" s="120" t="inlineStr">
+        <is>
+          <t>Маржа %</t>
+        </is>
+      </c>
+      <c r="F4" s="120" t="inlineStr">
+        <is>
+          <t>PB лет</t>
+        </is>
+      </c>
+      <c r="G4" s="120" t="inlineStr">
+        <is>
+          <t>NPV @10%</t>
+        </is>
+      </c>
+      <c r="H4" s="120" t="inlineStr">
+        <is>
+          <t>IRR %</t>
+        </is>
+      </c>
+      <c r="I4" s="120" t="inlineStr">
+        <is>
+          <t>Комментарий</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>База (II кв. 2026)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>5559.16</v>
+      </c>
+      <c r="C5" t="n">
+        <v>3342.93</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2216.23</v>
+      </c>
+      <c r="E5" s="121" t="n">
+        <v>0.399</v>
+      </c>
+      <c r="F5" t="n">
+        <v>5.41</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2253.2</v>
+      </c>
+      <c r="H5" s="121" t="n">
+        <v>0.1282</v>
+      </c>
+      <c r="I5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Яйцо −15%</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5397.88</v>
+      </c>
+      <c r="C6" t="n">
+        <v>3342.93</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2054.95</v>
+      </c>
+      <c r="E6" s="121" t="n">
+        <v>0.381</v>
+      </c>
+      <c r="F6" t="n">
+        <v>5.84</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1250.6</v>
+      </c>
+      <c r="H6" s="121" t="n">
+        <v>0.116</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>153,6 млн шт × 5,95 ₽</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Яйцо −30%</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>5236.6</v>
+      </c>
+      <c r="C7" t="n">
+        <v>3342.93</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1893.67</v>
+      </c>
+      <c r="E7" s="121" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="F7" t="n">
+        <v>6.34</v>
+      </c>
+      <c r="G7" t="n">
+        <v>248</v>
+      </c>
+      <c r="H7" s="121" t="n">
+        <v>0.1032</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>профицит рынка</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Корм +15%</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>5559.16</v>
+      </c>
+      <c r="C8" t="n">
+        <v>3623.12</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1936.04</v>
+      </c>
+      <c r="E8" s="121" t="n">
+        <v>0.348</v>
+      </c>
+      <c r="F8" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>511.4</v>
+      </c>
+      <c r="H8" s="121" t="n">
+        <v>0.1066</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>28 000 → 32 200 ₽/т</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Корм +20%</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>5559.16</v>
+      </c>
+      <c r="C9" t="n">
+        <v>3716.52</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1842.64</v>
+      </c>
+      <c r="E9" s="121" t="n">
+        <v>0.331</v>
+      </c>
+      <c r="F9" t="n">
+        <v>6.51</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-69.2</v>
+      </c>
+      <c r="H9" s="121" t="n">
+        <v>0.09910000000000001</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>стресс сырья</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Бройлер −10%</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>5210.17</v>
+      </c>
+      <c r="C10" t="n">
+        <v>3342.93</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1867.24</v>
+      </c>
+      <c r="E10" s="121" t="n">
+        <v>0.358</v>
+      </c>
+      <c r="F10" t="n">
+        <v>6.43</v>
+      </c>
+      <c r="G10" t="n">
+        <v>83.7</v>
+      </c>
+      <c r="H10" s="121" t="n">
+        <v>0.1011</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>205 → 184,5 ₽/кг</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ramp 85% (как 2029)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>4725.29</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2941.78</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1783.51</v>
+      </c>
+      <c r="E11" s="121" t="n">
+        <v>0.377</v>
+      </c>
+      <c r="F11" t="n">
+        <v>6.73</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-436.8</v>
+      </c>
+      <c r="H11" s="121" t="n">
+        <v>0.09420000000000001</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>выручка ×0,85; OPEX ×0,88 (часть постоянных)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Комбинированный стресс</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>5173.88</v>
+      </c>
+      <c r="C12" t="n">
+        <v>3623.12</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1550.76</v>
+      </c>
+      <c r="E12" s="121" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F12" t="n">
+        <v>7.74</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-1883.7</v>
+      </c>
+      <c r="H12" s="121" t="n">
+        <v>0.0741</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>яйцо −20%, бройлер −5%, корм +15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Оптимист (+5% цены мясо+яйцо)</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>5808.53</v>
+      </c>
+      <c r="C13" t="n">
+        <v>3342.93</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2465.6</v>
+      </c>
+      <c r="E13" s="121" t="n">
+        <v>0.424</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4.87</v>
+      </c>
+      <c r="G13" t="n">
+        <v>3803.4</v>
+      </c>
+      <c r="H13" s="121" t="n">
+        <v>0.1463</v>
+      </c>
+      <c r="I13" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="116" t="inlineStr">
+        <is>
+          <t>СЦЕНАРИИ ЭКСПОРТА (гипотезы)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Премия к выручке упрощённо: +3% на экспортный объём (логистика/FX не моделируются)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="118" t="inlineStr">
+        <is>
+          <t>Сценарий</t>
+        </is>
+      </c>
+      <c r="B4" s="118" t="inlineStr">
+        <is>
+          <t>Экспорт, млн ₽</t>
+        </is>
+      </c>
+      <c r="C4" s="118" t="inlineStr">
+        <is>
+          <t>Выручка итого</t>
+        </is>
+      </c>
+      <c r="D4" s="118" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="E4" s="118" t="inlineStr">
+        <is>
+          <t>NPV @10%</t>
+        </is>
+      </c>
+      <c r="F4" s="118" t="inlineStr">
+        <is>
+          <t>IRR %</t>
+        </is>
+      </c>
+      <c r="G4" s="118" t="inlineStr">
+        <is>
+          <t>Примечание</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Экспорт 0% (база)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>5559.2</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2216.2</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2253.2</v>
+      </c>
+      <c r="F5" s="121" t="n">
+        <v>0.1282</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>весь сбыт РФ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Экспорт 10% выручки</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>555.9</v>
+      </c>
+      <c r="C6" t="n">
+        <v>5575.8</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2232.9</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2356.8</v>
+      </c>
+      <c r="F6" s="121" t="n">
+        <v>0.1294</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>≈556 млн; без премии к цене</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Экспорт 15% только мясо</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>586.9</v>
+      </c>
+      <c r="C7" t="n">
+        <v>5576.8</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2233.8</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2362.6</v>
+      </c>
+      <c r="F7" s="121" t="n">
+        <v>0.1295</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>≈582 млн мяса</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Экспорт 20% мясо + премия 8%</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>845.1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>5584.5</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2241.6</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2410.8</v>
+      </c>
+      <c r="F8" s="121" t="n">
+        <v>0.1301</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>гипотеза MENA/СНГ</t>
         </is>
       </c>
     </row>
@@ -3211,7 +3819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="48" customWidth="1" style="58" min="1" max="1"/>
@@ -4483,23 +5091,23 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="58" t="inlineStr">
         <is>
           <t>Горизонт 2026–2035 · без долга · FCF = ЧП + амортизация · CAPEX в 2026</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="58" t="inlineStr">
         <is>
           <t>Ставка дисконтирования</t>
         </is>
       </c>
-      <c r="B3">
+      <c r="B3" s="58">
         <f>Допущения!C19</f>
         <v/>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="58" t="inlineStr">
         <is>
           <t>%</t>
         </is>
@@ -4558,657 +5166,657 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="58" t="n">
         <v>2026</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="58">
         <f>Экономика!B22</f>
         <v/>
       </c>
-      <c r="C6">
+      <c r="C6" s="58">
         <f>Экономика!B24</f>
         <v/>
       </c>
-      <c r="D6">
+      <c r="D6" s="58">
         <f>IF(B6&gt;0,Экономика!$B$9*B6,0)</f>
         <v/>
       </c>
-      <c r="E6">
+      <c r="E6" s="58">
         <f>C6-D6</f>
         <v/>
       </c>
-      <c r="F6">
+      <c r="F6" s="58">
         <f>MAX(E6*0.06,0)</f>
         <v/>
       </c>
-      <c r="G6">
+      <c r="G6" s="58">
         <f>E6-F6</f>
         <v/>
       </c>
-      <c r="H6">
+      <c r="H6" s="58">
         <f>G6+D6-Экономика!$B$4</f>
         <v/>
       </c>
-      <c r="I6">
+      <c r="I6" s="58">
         <f>1/(1+$B$3/100)^(6-5)</f>
         <v/>
       </c>
-      <c r="J6">
+      <c r="J6" s="58">
         <f>H6*I6</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="58" t="n">
         <v>2027</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="58">
         <f>Экономика!C22</f>
         <v/>
       </c>
-      <c r="C7">
+      <c r="C7" s="58">
         <f>Экономика!C24</f>
         <v/>
       </c>
-      <c r="D7">
+      <c r="D7" s="58">
         <f>IF(B7&gt;0,Экономика!$B$9*B7,0)</f>
         <v/>
       </c>
-      <c r="E7">
+      <c r="E7" s="58">
         <f>C7-D7</f>
         <v/>
       </c>
-      <c r="F7">
+      <c r="F7" s="58">
         <f>MAX(E7*0.06,0)</f>
         <v/>
       </c>
-      <c r="G7">
+      <c r="G7" s="58">
         <f>E7-F7</f>
         <v/>
       </c>
-      <c r="H7">
+      <c r="H7" s="58">
         <f>G7+D7</f>
         <v/>
       </c>
-      <c r="I7">
+      <c r="I7" s="58">
         <f>1/(1+$B$3/100)^(7-5)</f>
         <v/>
       </c>
-      <c r="J7">
+      <c r="J7" s="58">
         <f>H7*I7</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="58" t="n">
         <v>2028</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="58">
         <f>Экономика!D22</f>
         <v/>
       </c>
-      <c r="C8">
+      <c r="C8" s="58">
         <f>Экономика!D24</f>
         <v/>
       </c>
-      <c r="D8">
+      <c r="D8" s="58">
         <f>IF(B8&gt;0,Экономика!$B$9*B8,0)</f>
         <v/>
       </c>
-      <c r="E8">
+      <c r="E8" s="58">
         <f>C8-D8</f>
         <v/>
       </c>
-      <c r="F8">
+      <c r="F8" s="58">
         <f>MAX(E8*0.06,0)</f>
         <v/>
       </c>
-      <c r="G8">
+      <c r="G8" s="58">
         <f>E8-F8</f>
         <v/>
       </c>
-      <c r="H8">
+      <c r="H8" s="58">
         <f>G8+D8</f>
         <v/>
       </c>
-      <c r="I8">
+      <c r="I8" s="58">
         <f>1/(1+$B$3/100)^(8-5)</f>
         <v/>
       </c>
-      <c r="J8">
+      <c r="J8" s="58">
         <f>H8*I8</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="58" t="n">
         <v>2029</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="58">
         <f>Экономика!E22</f>
         <v/>
       </c>
-      <c r="C9">
+      <c r="C9" s="58">
         <f>Экономика!E24</f>
         <v/>
       </c>
-      <c r="D9">
+      <c r="D9" s="58">
         <f>IF(B9&gt;0,Экономика!$B$9*B9,0)</f>
         <v/>
       </c>
-      <c r="E9">
+      <c r="E9" s="58">
         <f>C9-D9</f>
         <v/>
       </c>
-      <c r="F9">
+      <c r="F9" s="58">
         <f>MAX(E9*0.06,0)</f>
         <v/>
       </c>
-      <c r="G9">
+      <c r="G9" s="58">
         <f>E9-F9</f>
         <v/>
       </c>
-      <c r="H9">
+      <c r="H9" s="58">
         <f>G9+D9</f>
         <v/>
       </c>
-      <c r="I9">
+      <c r="I9" s="58">
         <f>1/(1+$B$3/100)^(9-5)</f>
         <v/>
       </c>
-      <c r="J9">
+      <c r="J9" s="58">
         <f>H9*I9</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="58" t="n">
         <v>2030</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="58">
         <f>Экономика!F22</f>
         <v/>
       </c>
-      <c r="C10">
+      <c r="C10" s="58">
         <f>Экономика!F24</f>
         <v/>
       </c>
-      <c r="D10">
+      <c r="D10" s="58">
         <f>IF(B10&gt;0,Экономика!$B$9*B10,0)</f>
         <v/>
       </c>
-      <c r="E10">
+      <c r="E10" s="58">
         <f>C10-D10</f>
         <v/>
       </c>
-      <c r="F10">
+      <c r="F10" s="58">
         <f>MAX(E10*0.06,0)</f>
         <v/>
       </c>
-      <c r="G10">
+      <c r="G10" s="58">
         <f>E10-F10</f>
         <v/>
       </c>
-      <c r="H10">
+      <c r="H10" s="58">
         <f>G10+D10</f>
         <v/>
       </c>
-      <c r="I10">
+      <c r="I10" s="58">
         <f>1/(1+$B$3/100)^(10-5)</f>
         <v/>
       </c>
-      <c r="J10">
+      <c r="J10" s="58">
         <f>H10*I10</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="58" t="n">
         <v>2031</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="58">
         <f>Экономика!G22</f>
         <v/>
       </c>
-      <c r="C11">
+      <c r="C11" s="58">
         <f>Экономика!G24</f>
         <v/>
       </c>
-      <c r="D11">
+      <c r="D11" s="58">
         <f>IF(B11&gt;0,Экономика!$B$9*B11,0)</f>
         <v/>
       </c>
-      <c r="E11">
+      <c r="E11" s="58">
         <f>C11-D11</f>
         <v/>
       </c>
-      <c r="F11">
+      <c r="F11" s="58">
         <f>MAX(E11*0.06,0)</f>
         <v/>
       </c>
-      <c r="G11">
+      <c r="G11" s="58">
         <f>E11-F11</f>
         <v/>
       </c>
-      <c r="H11">
+      <c r="H11" s="58">
         <f>G11+D11</f>
         <v/>
       </c>
-      <c r="I11">
+      <c r="I11" s="58">
         <f>1/(1+$B$3/100)^(11-5)</f>
         <v/>
       </c>
-      <c r="J11">
+      <c r="J11" s="58">
         <f>H11*I11</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="58" t="n">
         <v>2032</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="58">
         <f>Экономика!H22</f>
         <v/>
       </c>
-      <c r="C12">
+      <c r="C12" s="58">
         <f>Экономика!H24</f>
         <v/>
       </c>
-      <c r="D12">
+      <c r="D12" s="58">
         <f>IF(B12&gt;0,Экономика!$B$9*B12,0)</f>
         <v/>
       </c>
-      <c r="E12">
+      <c r="E12" s="58">
         <f>C12-D12</f>
         <v/>
       </c>
-      <c r="F12">
+      <c r="F12" s="58">
         <f>MAX(E12*0.06,0)</f>
         <v/>
       </c>
-      <c r="G12">
+      <c r="G12" s="58">
         <f>E12-F12</f>
         <v/>
       </c>
-      <c r="H12">
+      <c r="H12" s="58">
         <f>G12+D12</f>
         <v/>
       </c>
-      <c r="I12">
+      <c r="I12" s="58">
         <f>1/(1+$B$3/100)^(12-5)</f>
         <v/>
       </c>
-      <c r="J12">
+      <c r="J12" s="58">
         <f>H12*I12</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" s="58" t="n">
         <v>2033</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="58">
         <f>Экономика!I22</f>
         <v/>
       </c>
-      <c r="C13">
+      <c r="C13" s="58">
         <f>Экономика!I24</f>
         <v/>
       </c>
-      <c r="D13">
+      <c r="D13" s="58">
         <f>IF(B13&gt;0,Экономика!$B$9*B13,0)</f>
         <v/>
       </c>
-      <c r="E13">
+      <c r="E13" s="58">
         <f>C13-D13</f>
         <v/>
       </c>
-      <c r="F13">
+      <c r="F13" s="58">
         <f>MAX(E13*0.06,0)</f>
         <v/>
       </c>
-      <c r="G13">
+      <c r="G13" s="58">
         <f>E13-F13</f>
         <v/>
       </c>
-      <c r="H13">
+      <c r="H13" s="58">
         <f>G13+D13</f>
         <v/>
       </c>
-      <c r="I13">
+      <c r="I13" s="58">
         <f>1/(1+$B$3/100)^(13-5)</f>
         <v/>
       </c>
-      <c r="J13">
+      <c r="J13" s="58">
         <f>H13*I13</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="58" t="n">
         <v>2034</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="58">
         <f>Экономика!J22</f>
         <v/>
       </c>
-      <c r="C14">
+      <c r="C14" s="58">
         <f>Экономика!J24</f>
         <v/>
       </c>
-      <c r="D14">
+      <c r="D14" s="58">
         <f>IF(B14&gt;0,Экономика!$B$9*B14,0)</f>
         <v/>
       </c>
-      <c r="E14">
+      <c r="E14" s="58">
         <f>C14-D14</f>
         <v/>
       </c>
-      <c r="F14">
+      <c r="F14" s="58">
         <f>MAX(E14*0.06,0)</f>
         <v/>
       </c>
-      <c r="G14">
+      <c r="G14" s="58">
         <f>E14-F14</f>
         <v/>
       </c>
-      <c r="H14">
+      <c r="H14" s="58">
         <f>G14+D14</f>
         <v/>
       </c>
-      <c r="I14">
+      <c r="I14" s="58">
         <f>1/(1+$B$3/100)^(14-5)</f>
         <v/>
       </c>
-      <c r="J14">
+      <c r="J14" s="58">
         <f>H14*I14</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" s="58" t="n">
         <v>2035</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="58">
         <f>Экономика!K22</f>
         <v/>
       </c>
-      <c r="C15">
+      <c r="C15" s="58">
         <f>Экономика!K24</f>
         <v/>
       </c>
-      <c r="D15">
+      <c r="D15" s="58">
         <f>IF(B15&gt;0,Экономика!$B$9*B15,0)</f>
         <v/>
       </c>
-      <c r="E15">
+      <c r="E15" s="58">
         <f>C15-D15</f>
         <v/>
       </c>
-      <c r="F15">
+      <c r="F15" s="58">
         <f>MAX(E15*0.06,0)</f>
         <v/>
       </c>
-      <c r="G15">
+      <c r="G15" s="58">
         <f>E15-F15</f>
         <v/>
       </c>
-      <c r="H15">
+      <c r="H15" s="58">
         <f>G15+D15</f>
         <v/>
       </c>
-      <c r="I15">
+      <c r="I15" s="58">
         <f>1/(1+$B$3/100)^(15-5)</f>
         <v/>
       </c>
-      <c r="J15">
+      <c r="J15" s="58">
         <f>H15*I15</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="58" t="n">
         <v>2036</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="58">
         <f>1</f>
         <v/>
       </c>
-      <c r="C16">
+      <c r="C16" s="58">
         <f>Экономика!$B$7</f>
         <v/>
       </c>
-      <c r="D16">
+      <c r="D16" s="58">
         <f>IF(B16&gt;0,Экономика!$B$9*B16,0)</f>
         <v/>
       </c>
-      <c r="E16">
+      <c r="E16" s="58">
         <f>C16-D16</f>
         <v/>
       </c>
-      <c r="F16">
+      <c r="F16" s="58">
         <f>MAX(E16*0.06,0)</f>
         <v/>
       </c>
-      <c r="G16">
+      <c r="G16" s="58">
         <f>E16-F16</f>
         <v/>
       </c>
-      <c r="H16">
+      <c r="H16" s="58">
         <f>G16+D16</f>
         <v/>
       </c>
-      <c r="I16">
+      <c r="I16" s="58">
         <f>1/(1+$B$3/100)^(16-5)</f>
         <v/>
       </c>
-      <c r="J16">
+      <c r="J16" s="58">
         <f>H16*I16</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="58" t="n">
         <v>2037</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="58">
         <f>1</f>
         <v/>
       </c>
-      <c r="C17">
+      <c r="C17" s="58">
         <f>Экономика!$B$7</f>
         <v/>
       </c>
-      <c r="D17">
+      <c r="D17" s="58">
         <f>IF(B17&gt;0,Экономика!$B$9*B17,0)</f>
         <v/>
       </c>
-      <c r="E17">
+      <c r="E17" s="58">
         <f>C17-D17</f>
         <v/>
       </c>
-      <c r="F17">
+      <c r="F17" s="58">
         <f>MAX(E17*0.06,0)</f>
         <v/>
       </c>
-      <c r="G17">
+      <c r="G17" s="58">
         <f>E17-F17</f>
         <v/>
       </c>
-      <c r="H17">
+      <c r="H17" s="58">
         <f>G17+D17</f>
         <v/>
       </c>
-      <c r="I17">
+      <c r="I17" s="58">
         <f>1/(1+$B$3/100)^(17-5)</f>
         <v/>
       </c>
-      <c r="J17">
+      <c r="J17" s="58">
         <f>H17*I17</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
+      <c r="A18" s="58" t="n">
         <v>2038</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="58">
         <f>1</f>
         <v/>
       </c>
-      <c r="C18">
+      <c r="C18" s="58">
         <f>Экономика!$B$7</f>
         <v/>
       </c>
-      <c r="D18">
+      <c r="D18" s="58">
         <f>IF(B18&gt;0,Экономика!$B$9*B18,0)</f>
         <v/>
       </c>
-      <c r="E18">
+      <c r="E18" s="58">
         <f>C18-D18</f>
         <v/>
       </c>
-      <c r="F18">
+      <c r="F18" s="58">
         <f>MAX(E18*0.06,0)</f>
         <v/>
       </c>
-      <c r="G18">
+      <c r="G18" s="58">
         <f>E18-F18</f>
         <v/>
       </c>
-      <c r="H18">
+      <c r="H18" s="58">
         <f>G18+D18</f>
         <v/>
       </c>
-      <c r="I18">
+      <c r="I18" s="58">
         <f>1/(1+$B$3/100)^(18-5)</f>
         <v/>
       </c>
-      <c r="J18">
+      <c r="J18" s="58">
         <f>H18*I18</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
+      <c r="A19" s="58" t="n">
         <v>2039</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="58">
         <f>1</f>
         <v/>
       </c>
-      <c r="C19">
+      <c r="C19" s="58">
         <f>Экономика!$B$7</f>
         <v/>
       </c>
-      <c r="D19">
+      <c r="D19" s="58">
         <f>IF(B19&gt;0,Экономика!$B$9*B19,0)</f>
         <v/>
       </c>
-      <c r="E19">
+      <c r="E19" s="58">
         <f>C19-D19</f>
         <v/>
       </c>
-      <c r="F19">
+      <c r="F19" s="58">
         <f>MAX(E19*0.06,0)</f>
         <v/>
       </c>
-      <c r="G19">
+      <c r="G19" s="58">
         <f>E19-F19</f>
         <v/>
       </c>
-      <c r="H19">
+      <c r="H19" s="58">
         <f>G19+D19</f>
         <v/>
       </c>
-      <c r="I19">
+      <c r="I19" s="58">
         <f>1/(1+$B$3/100)^(19-5)</f>
         <v/>
       </c>
-      <c r="J19">
+      <c r="J19" s="58">
         <f>H19*I19</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" s="58" t="n">
         <v>2040</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="58">
         <f>1</f>
         <v/>
       </c>
-      <c r="C20">
+      <c r="C20" s="58">
         <f>Экономика!$B$7</f>
         <v/>
       </c>
-      <c r="D20">
+      <c r="D20" s="58">
         <f>IF(B20&gt;0,Экономика!$B$9*B20,0)</f>
         <v/>
       </c>
-      <c r="E20">
+      <c r="E20" s="58">
         <f>C20-D20</f>
         <v/>
       </c>
-      <c r="F20">
+      <c r="F20" s="58">
         <f>MAX(E20*0.06,0)</f>
         <v/>
       </c>
-      <c r="G20">
+      <c r="G20" s="58">
         <f>E20-F20</f>
         <v/>
       </c>
-      <c r="H20">
+      <c r="H20" s="58">
         <f>G20+D20</f>
         <v/>
       </c>
-      <c r="I20">
+      <c r="I20" s="58">
         <f>1/(1+$B$3/100)^(20-5)</f>
         <v/>
       </c>
-      <c r="J20">
+      <c r="J20" s="58">
         <f>H20*I20</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" s="58" t="n">
         <v>2041</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="58">
         <f>1</f>
         <v/>
       </c>
-      <c r="C21">
+      <c r="C21" s="58">
         <f>Экономика!$B$7</f>
         <v/>
       </c>
-      <c r="D21">
+      <c r="D21" s="58">
         <f>IF(B21&gt;0,Экономика!$B$9*B21,0)</f>
         <v/>
       </c>
-      <c r="E21">
+      <c r="E21" s="58">
         <f>C21-D21</f>
         <v/>
       </c>
-      <c r="F21">
+      <c r="F21" s="58">
         <f>MAX(E21*0.06,0)</f>
         <v/>
       </c>
-      <c r="G21">
+      <c r="G21" s="58">
         <f>E21-F21</f>
         <v/>
       </c>
-      <c r="H21">
+      <c r="H21" s="58">
         <f>G21+D21</f>
         <v/>
       </c>
-      <c r="I21">
+      <c r="I21" s="58">
         <f>1/(1+$B$3/100)^(21-5)</f>
         <v/>
       </c>
-      <c r="J21">
+      <c r="J21" s="58">
         <f>H21*I21</f>
         <v/>
       </c>
@@ -5219,7 +5827,7 @@
           <t>NPV @ 10%, млн ₽</t>
         </is>
       </c>
-      <c r="B22">
+      <c r="B22" s="58">
         <f>SUM(J6:J21)</f>
         <v/>
       </c>
@@ -5230,7 +5838,7 @@
           <t>IRR, %</t>
         </is>
       </c>
-      <c r="B23">
+      <c r="B23" s="58">
         <f>IRR(H6:H21)*100</f>
         <v/>
       </c>
@@ -5241,30 +5849,30 @@
           <t>PI (NPV/CAPEX + 1)</t>
         </is>
       </c>
-      <c r="B24">
+      <c r="B24" s="58">
         <f>B22/Экономика!B4+1</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="58" t="inlineStr">
         <is>
           <t>Сравнение с кроликами (docx tab#7)</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="58" t="inlineStr">
         <is>
           <t>Кролики NPV @ 10%</t>
         </is>
       </c>
-      <c r="B27" t="n">
+      <c r="B27" s="58" t="n">
         <v>2779.5</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="58" t="inlineStr">
         <is>
           <t>Кролики IRR</t>
         </is>
@@ -5274,12 +5882,12 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="58" t="inlineStr">
         <is>
           <t>Горизонт DCF</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="58" t="inlineStr">
         <is>
           <t>16 лет (2026–2041)</t>
         </is>

</xml_diff>

<commit_message>
Fix export NPV (honest: slightly negative at 6% meat) and calc script
Co-authored-by: Demid369 <Demid369@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/teo-poultry/_incoming/finmodel-pticekompleks-12-mlrd.xlsx
+++ b/docs/teo-poultry/_incoming/finmodel-pticekompleks-12-mlrd.xlsx
@@ -2366,7 +2366,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Экспорт 0% (база)</t>
+          <t>Экспорт 0% (база finmodel)</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -2393,81 +2393,81 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Экспорт 10% выручки</t>
+          <t>План 6% мяса, дружественные страны</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>555.9</v>
+        <v>234.7</v>
       </c>
       <c r="C6" t="n">
-        <v>5575.8</v>
+        <v>5563.9</v>
       </c>
       <c r="D6" t="n">
-        <v>2232.9</v>
+        <v>2209.9</v>
       </c>
       <c r="E6" t="n">
-        <v>2356.8</v>
+        <v>2214</v>
       </c>
       <c r="F6" s="121" t="n">
-        <v>0.1294</v>
+        <v>0.1277</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>≈556 млн; без премии к цене</t>
+          <t>235 млн ₽; KZ/UZ/BY/IR/KG/AE/AM/EG/AZ; год 4+</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Экспорт 15% только мясо</t>
+          <t>Экспорт 10% выручки (стресс-тест)</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>586.9</v>
+        <v>555.9</v>
       </c>
       <c r="C7" t="n">
-        <v>5576.8</v>
+        <v>5575.8</v>
       </c>
       <c r="D7" t="n">
-        <v>2233.8</v>
+        <v>2214.9</v>
       </c>
       <c r="E7" t="n">
-        <v>2362.6</v>
+        <v>2245</v>
       </c>
       <c r="F7" s="121" t="n">
-        <v>0.1295</v>
+        <v>0.1281</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>≈582 млн мяса</t>
+          <t>агрессивный; не базовый план</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Экспорт 20% мясо + премия 8%</t>
+          <t>Экспорт 15% только мясо (стресс-тест)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>845.1</v>
+        <v>586.9</v>
       </c>
       <c r="C8" t="n">
-        <v>5584.5</v>
+        <v>5576.8</v>
       </c>
       <c r="D8" t="n">
-        <v>2241.6</v>
+        <v>2211.8</v>
       </c>
       <c r="E8" t="n">
-        <v>2410.8</v>
+        <v>2225.9</v>
       </c>
       <c r="F8" s="121" t="n">
-        <v>0.1301</v>
+        <v>0.1279</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>гипотеза MENA/СНГ</t>
+          <t>верхняя граница при перепроизводстве</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Export: move APK Tab#5 10.2 bln to poultry block; zero poultry product export
Co-authored-by: Demid369 <Demid369@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/teo-poultry/_incoming/finmodel-pticekompleks-12-mlrd.xlsx
+++ b/docs/teo-poultry/_incoming/finmodel-pticekompleks-12-mlrd.xlsx
@@ -2309,20 +2309,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="116" t="inlineStr">
         <is>
-          <t>СЦЕНАРИИ ЭКСПОРТА (гипотезы)</t>
+          <t>ЭКСПОРТ — Tab#5 baseline на блок 1</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Премия к выручке упрощённо: +3% на экспортный объём (логистика/FX не моделируются)</t>
+          <t>Птица: 0% export (finmodel 5 559 РФ). APK 10 208 млн — consolidated, вне NPV 12 млрд</t>
         </is>
       </c>
     </row>
@@ -2339,7 +2339,7 @@
       </c>
       <c r="C4" s="118" t="inlineStr">
         <is>
-          <t>Выручка итого</t>
+          <t>Выручка finmodel</t>
         </is>
       </c>
       <c r="D4" s="118" t="inlineStr">
@@ -2366,7 +2366,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Экспорт 0% (база finmodel)</t>
+          <t>Птица: весь сбыт РФ (finmodel)</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -2386,88 +2386,82 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>весь сбыт РФ</t>
+          <t>мясо, яйцо, удобрение — 0% export</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>План 6% мяса, дружественные страны</t>
+          <t>APK Tab#5: Натуральная кожа (КРС+МРС)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>234.7</v>
-      </c>
-      <c r="C6" t="n">
-        <v>5563.9</v>
-      </c>
-      <c r="D6" t="n">
-        <v>2209.9</v>
-      </c>
-      <c r="E6" t="n">
-        <v>2214</v>
-      </c>
-      <c r="F6" s="121" t="n">
-        <v>0.1277</v>
+        <v>1478.5</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>235 млн ₽; KZ/UZ/BY/IR/KG/AE/AM/EG/AZ; год 4+</t>
+          <t>consolidated APK; не в NPV finmodel 12 млрд</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Экспорт 10% выручки (стресс-тест)</t>
+          <t>APK Tab#5: Желатин халяльный</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>555.9</v>
-      </c>
-      <c r="C7" t="n">
-        <v>5575.8</v>
-      </c>
-      <c r="D7" t="n">
-        <v>2214.9</v>
-      </c>
-      <c r="E7" t="n">
-        <v>2245</v>
-      </c>
-      <c r="F7" s="121" t="n">
-        <v>0.1281</v>
+        <v>3840</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>агрессивный; не базовый план</t>
+          <t>consolidated APK; не в NPV finmodel 12 млрд</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Экспорт 15% только мясо (стресс-тест)</t>
+          <t>APK Tab#5: Шерсть овец</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>586.9</v>
-      </c>
-      <c r="C8" t="n">
-        <v>5576.8</v>
-      </c>
-      <c r="D8" t="n">
-        <v>2211.8</v>
-      </c>
-      <c r="E8" t="n">
-        <v>2225.9</v>
-      </c>
-      <c r="F8" s="121" t="n">
-        <v>0.1279</v>
+        <v>90</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>верхняя граница при перепроизводстве</t>
+          <t>consolidated APK; не в NPV finmodel 12 млрд</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>APK Tab#5: Чёрная икра белуги</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>4800</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>consolidated APK; не в NPV finmodel 12 млрд</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ИТОГО APK экспорт (блок 1)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>10208.5</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>10 208 млн ≈ 10,2 млрд; export-apk-baseline-tab5.md</t>
         </is>
       </c>
     </row>

</xml_diff>